<commit_message>
add lab 12 rubric and update schedule
</commit_message>
<xml_diff>
--- a/syllabus/class_schedule.xlsx
+++ b/syllabus/class_schedule.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10208"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10404"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/judebayham/Documents/git_projects/arec-330/syllabus/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54A98D42-4F01-5548-9742-1B601637C869}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A89B706-442A-2F4A-9A11-40DD9AF172C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="12020" yWindow="680" windowWidth="17920" windowHeight="20320" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -120,9 +120,6 @@
     <t>Storytelling with data</t>
   </si>
   <si>
-    <t>Understand the Context</t>
-  </si>
-  <si>
     <t>Choose Visual</t>
   </si>
   <si>
@@ -178,6 +175,9 @@
   </si>
   <si>
     <t>Forecasting (asynchronous)</t>
+  </si>
+  <si>
+    <t>Project Proposal</t>
   </si>
 </sst>
 </file>
@@ -624,7 +624,7 @@
         <v>5</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E2" s="2"/>
     </row>
@@ -637,7 +637,7 @@
         <v>46050</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D3" t="s">
         <v>6</v>
@@ -653,7 +653,7 @@
         <v>46057</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D4" t="s">
         <v>7</v>
@@ -669,10 +669,10 @@
         <v>46064</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="13" x14ac:dyDescent="0.15">
@@ -687,7 +687,7 @@
         <v>8</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E6" s="2"/>
     </row>
@@ -700,7 +700,7 @@
         <v>46078</v>
       </c>
       <c r="C7" s="12" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D7" s="8" t="s">
         <v>9</v>
@@ -715,7 +715,7 @@
         <v>46085</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D8" t="s">
         <v>10</v>
@@ -731,7 +731,7 @@
         <v>46092</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D9" t="s">
         <v>11</v>
@@ -747,7 +747,7 @@
         <v>46099</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D10" s="9"/>
       <c r="E10" s="2"/>
@@ -778,8 +778,8 @@
       <c r="C12" t="s">
         <v>14</v>
       </c>
-      <c r="D12" t="s">
-        <v>15</v>
+      <c r="D12" s="5" t="s">
+        <v>34</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="13" x14ac:dyDescent="0.15">
@@ -791,10 +791,10 @@
         <v>46120</v>
       </c>
       <c r="C13" t="s">
+        <v>15</v>
+      </c>
+      <c r="D13" t="s">
         <v>16</v>
-      </c>
-      <c r="D13" t="s">
-        <v>17</v>
       </c>
       <c r="E13" s="6"/>
     </row>
@@ -807,10 +807,10 @@
         <v>46127</v>
       </c>
       <c r="C14" t="s">
+        <v>17</v>
+      </c>
+      <c r="D14" s="8" t="s">
         <v>18</v>
-      </c>
-      <c r="D14" s="8" t="s">
-        <v>19</v>
       </c>
       <c r="E14" s="2"/>
     </row>
@@ -823,10 +823,10 @@
         <v>46134</v>
       </c>
       <c r="C15" t="s">
+        <v>19</v>
+      </c>
+      <c r="D15" t="s">
         <v>20</v>
-      </c>
-      <c r="D15" t="s">
-        <v>21</v>
       </c>
       <c r="E15" s="5"/>
     </row>
@@ -839,10 +839,10 @@
         <v>46141</v>
       </c>
       <c r="C16" t="s">
+        <v>21</v>
+      </c>
+      <c r="D16" s="8" t="s">
         <v>22</v>
-      </c>
-      <c r="D16" s="8" t="s">
-        <v>23</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="13" x14ac:dyDescent="0.15">
@@ -854,10 +854,10 @@
         <v>46148</v>
       </c>
       <c r="C17" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D17" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E17" s="2"/>
     </row>

</xml_diff>